<commit_message>
docs: Upgrade Excel tracking to Enterprise-Level documentation standard
</commit_message>
<xml_diff>
--- a/docs/Git_Push_History.xlsx
+++ b/docs/Git_Push_History.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,47 +441,57 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Git Push ID</t>
+          <t>Version (Major.Minor.Build)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Git Push ID / Commit Hash</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Module</t>
+          <t>Affected Module / Workflow</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Change Summary</t>
+          <t>What was changed</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Detailed Changes</t>
+          <t>Why it was changed</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Bugs Fixed</t>
+          <t>How it works now</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Features Added</t>
+          <t>Bugs / Issues Fixed</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>New Functionality Added</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>What was tested</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Current Status</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Limitations / Pending Work</t>
         </is>
       </c>
     </row>
@@ -498,14 +508,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>5.0.2</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>5278463</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>5.0.2</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>Backend (RAG Engine)</t>
@@ -513,34 +523,40 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Updated the intent router to strip conversational fluff like "where is" to properly extract book titles. Removed hardcoded entrance fallback so the system forcefully prompts users for their location before initiating a route.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>Fixed catalog search bug and updated location routing logic.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Updated the intent router to strip conversational fluff like "where is" to properly extract book titles. Removed hardcoded entrance fallback so the system forcefully prompts users for their location before initiating a route.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Fixed catalog lookup failing on "where is" questions.</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Interactive 2-step location routing.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Tested on local backend.</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Deployed</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -555,14 +571,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>5.0.3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>20f9216</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>5.0.3</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>Frontend (Wayfinder)</t>
@@ -570,30 +586,36 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>Replaced generic guidance with a mathematical heading vector system that calculates cross-products of movement vectors to accurately instruct users to Turn left, Turn right, or Head straight.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>Added GPS-style turn-by-turn navigation.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Replaced generic guidance with a mathematical heading vector system that calculates cross-products of movement vectors to accurately instruct users to Turn left, Turn right, or Head straight.</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
         <is>
           <t>Precise directional turn-by-turn logic.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Verified grid traversal cross products.</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Deployed</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -608,14 +630,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>5.0.4</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>df2830d</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>5.0.4</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>Frontend (Voice Assistant)</t>
@@ -623,30 +645,36 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>Updated the fullscreen map UI to dynamically read the admin architecture configuration and render buttons for all active floors rather than being hardcoded to just Floor 1 and 2.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>Dynamic floor switcher buttons in 3D Map.</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Updated the fullscreen map UI to dynamically read the admin architecture configuration and render buttons for all active floors rather than being hardcoded to just Floor 1 and 2.</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>Dynamic floor synchronization.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Verified UI button generation.</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Deployed</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -661,14 +689,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>5.0.5</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>45dda18</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>5.0.5</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>Backend (LLM Config)</t>
@@ -676,30 +704,36 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>Updated GROQ_MODEL in config.py from llama-3.1-8b-instant (which returned 404) to llama3-8b-8192 to resolve API failures.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>Changed Groq Model ID.</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Updated GROQ_MODEL in config.py from llama-3.1-8b-instant (which returned 404) to llama3-8b-8192 to resolve API failures.</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Fixed 404 Model Not Found error on Groq.</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
         <is>
           <t>Tested connection logic.</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Superseded</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -714,14 +748,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>5.0.6</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>295b9bd</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>5.0.6</t>
-        </is>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>Frontend &amp; Backend</t>
@@ -729,30 +763,36 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>Removed onConfigLoaded from LibraryWayfinder useEffect dependencies to stop an infinite fetch loop when the session expired. Changed Groq model to mixtral-8x7b-32768 after discovering llama3-8b-8192 was decommissioned.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>Fixed WebGL leak and updated Groq model.</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Removed onConfigLoaded from LibraryWayfinder useEffect dependencies to stop an infinite fetch loop when the session expired. Changed Groq model to mixtral-8x7b-32768 after discovering llama3-8b-8192 was decommissioned.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Fixed "Too many active WebGL contexts" memory leak. Fixed Groq 400 decommission error.</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
         <is>
           <t>Verified infinite loop fix in useEffect.</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Superseded</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -767,14 +807,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>5.0.7</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>90f719b</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>5.0.7</t>
-        </is>
-      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>Backend (LLM Config)</t>
@@ -782,30 +822,36 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>Wrote a script to query the allowed models on the user's specific Groq API key tier, and updated config.py to use qwen/qwen3.6-27b which was confirmed to work and support thinking blocks.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
           <t>Final Groq Model alignment for API key.</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Wrote a script to query the allowed models on the user's specific Groq API key tier, and updated config.py to use qwen/qwen3.6-27b which was confirmed to work and support thinking blocks.</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Fixed 403 / 400 errors across all standard models for this specific API key.</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
         <is>
           <t>Tested API key capabilities via Python urllib script.</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Live / Deployed</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update enterprise tracking logs for v5.1.0
</commit_message>
<xml_diff>
--- a/docs/Git_Push_History.xlsx
+++ b/docs/Git_Push_History.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:V8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,6 +494,51 @@
           <t>Limitations / Pending Work</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Git Push ID</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Change Summary</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Detailed Changes</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Bugs Fixed</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Features Added</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -557,6 +602,15 @@
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -616,6 +670,15 @@
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -675,6 +738,15 @@
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -734,6 +806,15 @@
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -793,6 +874,15 @@
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -852,6 +942,83 @@
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>09:59</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>237b894</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>5.1.0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Admin Panel &amp; RAG Engine</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Completed Books API, Analytics Dashboard, and Real-time SQL Sync</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Created fully working Books API so Admin UI can Add/Edit/Delete books. Added AI Chat Audit Log and Analytics Dashboard (showing Top Missing Books). Modified the RAG search engine to directly query the live SQLite database first, bypassing ChromaDB for exact titles, which fixes the stale data bug and drops search latency to milliseconds. Added time-based Voice Assistant greeting.</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Fixed stale book location data by querying live DB. Reduced agent latency. Added missing Voice greeting.</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Analytics Page, AI Chat Audit Logs, Time-based Mic Greeting.</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Verified SQL query execution in search_catalog.</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Live / Deployed</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Version 5.2.0: Settings Module Phase 3
</commit_message>
<xml_diff>
--- a/docs/Git_Push_History.xlsx
+++ b/docs/Git_Push_History.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1020,6 +1020,70 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10:06</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>5.2.0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Admin Panel (Settings)</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Completed Phase 3: Global Library Settings Injection</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Added library_name, opening_hours, and library_policies to the LibraryConfig database schema. Built the Settings.jsx UI panel for admins to edit these fields. Modified the core AI RAG engine (engine.py) to dynamically query these settings from the live database and inject them directly into the LLM System Prompt. The Voice AI will now enforce custom library rules globally.</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Dynamic Library Settings UI, AI System Prompt Injection.</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Verified UI saves correctly to DB and engine retrieves it.</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Live / Deployed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update enterprise tracking logs for v5.3.0
</commit_message>
<xml_diff>
--- a/docs/Git_Push_History.xlsx
+++ b/docs/Git_Push_History.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1084,6 +1084,70 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10:14</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>4b71756</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>5.3.0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Admin Panel (Users &amp; Departments)</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Completed Phase 4: Users and Departments Management</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Added a Create User modal to Users.jsx allowing Admins to register new users or other admins. Verified that Departments.jsx is fully functional for tracking campus buildings, HODs, and floors.</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Admin user creation capability.</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Verified UI rendering.</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Live / Deployed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update enterprise tracking logs for v6.0.0
</commit_message>
<xml_diff>
--- a/docs/Git_Push_History.xlsx
+++ b/docs/Git_Push_History.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V10"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1148,6 +1148,70 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>9173e3f</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>6.0.0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>V6.0 Experience Upgrades</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Completed Phase 6, 7, 8, 9</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Verified Text Chat UI functionality. Added AI Voice preset customization (Aria, Guy, Sonia, Neerja, Natasha) to the database and Settings.jsx. Integrated selected voice with edge-tts in main.py. Added an animated dashed texture effect to the 3D map route line in LibraryWayfinder.jsx. Added an Export CSV button to Analytics.jsx to download missing books data.</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Voice Selection dropdown, Animated Map Paths, Analytics CSV Export.</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Verified UI rendering.</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Live / Deployed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>